<commit_message>
Re-lock paper set on 27 Sep 2026 register and method update
Lifetime 7,167.1 -> 7,390.3 MtCO2e.
Peak 235.9 -> 253.4 MtCO2e in 2037.
Damages C$3,106 bn -> C$3,176 bn.
NPV C$1,945 bn -> C$2,015 bn.
Export capacity 79.6 -> 85.55 mtpa.
Paper-set SHA-256 94f7042ab86e6aa87091b26fdac35ebc0af7b5ad28dc05c9a5f6f135de8a69c3 -> 77d14a4b9f7ae2cc5225a4c4019aba5839c8f4e613dbc911de3d12c96d8d21f9.
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Data_Inputs.xlsx
+++ b/Inputs/Canada_LNG_Data_Inputs.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20 10:00 UTC</t>
+          <t>2026-09-27 (inputs update; see Emission Factors liquefaction and Parameters fid_delay_mid)</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Each stage carries a single central figure. Low and high are recorded for reference and are not used to build scenarios. The stages are not correlated: combustion varies by about 9 per cent with gas composition, while upstream varies by a factor of three because measurement is difficult. Moving all six together would produce a spread wider than anything physically plausible.</t>
+          <t>Each stage carries a single central figure. Low and high are not used to build scenarios; they set the triangle each stage is sampled on in the Monte Carlo. The stages are not correlated: combustion varies by about 9 per cent with gas composition, while upstream varies by a factor of three because measurement is difficult. Moving all six together would produce a spread wider than anything physically plausible.</t>
         </is>
       </c>
     </row>
@@ -758,12 +758,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Liquefaction is a single central value</t>
+          <t>Liquefaction: one central value, gas-turbine range</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>The liquefaction stage carries a central factor of 0.29 tCO2e per tonne (gas turbine) for every terminal and its whole operating life. 0.12 is kept as range_low and applies only if electrification is contracted and delivered. Electric drive is not assumed for any project.</t>
+          <t>The liquefaction stage carries a central factor of 0.29 tCO2e per tonne (gas turbine) for every terminal and its whole operating life. The Monte Carlo samples 0.26 / 0.29 / 0.36, the range for gas-turbine plants in Delphi Group (2013) (Sabine Pass 0.26, Pluto 0.36). Electric drive is not assumed for any project; it is a separate sensitivity with every terminal electric at 0.15 (Pembina, Gorski and Lam 2023) and 0.021 (BC EAO, Ksi Lisims grid case). The two together show all gas against all electric.</t>
         </is>
       </c>
     </row>
@@ -1047,6 +1047,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
@@ -1244,7 +1245,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Gas is chilled to minus 162 degrees at the terminal until it becomes liquid. Energy intensive. The central factor is gas-turbine drive for every terminal; electric-drive 0.12 is retained only as range_low.</t>
+          <t>Gas is chilled to minus 162 degrees at the terminal until it becomes liquid. Energy intensive. The central factor is gas-turbine drive for every terminal. The Monte Carlo samples 0.26 to 0.36, the range for gas-turbine plants. Electric drive is not in this range: it is a separate sensitivity with every terminal electric (Parameters liquefaction_electric 0.15 and liquefaction_electric_drive_grid 0.021).</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1261,7 +1262,7 @@
         <v>0.29</v>
       </c>
       <c r="F4" t="n">
-        <v>0.15</v>
+        <v>0.26</v>
       </c>
       <c r="G4" t="n">
         <v>0.36</v>
@@ -1273,7 +1274,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>range_low 0.15 tCO2e per t LNG: Pembina Institute, Squaring the Circle: State of LNG 2023, https://www.pembina.org/reports/squaring-the-circle-state-of-lng-2023.pdf , reported figure for LNG Canada Phase 1 under electric drive. Adopted 3 September 2026, replacing 0.12, which no Pembina document states and which appears to have been a misreading of the 0.11 tCO2e/t REDUCTION reported in Wellhead to Waterline (2014) as an absolute intensity. The same Pembina report gives 0.059 for LNG Canada Phase 2 and 0.04 for Woodfibre; those are facility-specific and are not used. range_low is a counterfactual for the figure-8 appendix only and is not used in the central case. range_high 0.36 remains an uncited literature upper bound for gas-turbine plants. Corroboration on the central: IEA (2025), page 13, gives a global average liquefaction intensity of about 6 g CO2-eq/MJ of LNG, which at 55 MJ/kg is 0.33 tCO2e/t - above this model's 0.29, so 0.29 is not a high-side choice. https://iea.blob.core.windows.net/assets/df9b1bed-4e16-4db8-bec5-a5fa117a9130/AssessingemissionsfromLNGsupplyandabatementoptions.pdf</t>
+          <t>Both ends are gas-turbine plants in Delphi Group (2013), LNG Emissions Benchmarking, prepared for the BC Ministry of Environment, March 2013: https://www2.gov.bc.ca/assets/gov/environment/climate-change/ind/lng/lng_emissions_benchmarking_-_march_2013.pdf . range_low 0.26 tCO2e per t LNG: Sabine Pass, the lowest gas-turbine plant in the benchmark (page 23, Figure 3). Adopted 27 September 2026, replacing 0.15. range_high 0.36 tCO2e per t LNG: Pluto LNG, a gas-turbine plant (GE Frame 7EA), in a benchmark of operating and proposed plants that ranged from 0.17 to 0.49 (page 14). Cited 27 September 2026; previously an uncited literature upper bound. The Monte Carlo samples liquefaction on the triangle 0.26 / 0.29 / 0.36 from 27 September 2026 (decision: Freddie). Electric drive is deliberately outside this range. The former range_low 0.15 (Pembina Institute, Gorski and Lam 2023, Squaring the Circle: State of LNG 2023, https://www.pembina.org/reports/squaring-the-circle-state-of-lng-2023.pdf , LNG Canada under electric drive) now lives only on the Parameters sheet as liquefaction_electric and drives the all-electric sensitivity in src/drive_sensitivity.py. Corroboration on the central: IEA (2025), page 13, gives a global average liquefaction intensity of about 6 g CO2-eq/MJ of LNG, which at 55 MJ/kg is 0.33 tCO2e/t - above this model's 0.29, so 0.29 is not a high-side choice. https://iea.blob.core.windows.net/assets/df9b1bed-4e16-4db8-bec5-a5fa117a9130/AssessingemissionsfromLNGsupplyandabatementoptions.pdf</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -1890,7 +1891,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Unchanged at 5, so the central case is untouched by the 3 September 2026 band change. Applied to the seven proposed assets without FID. post_fid_to_completion = 4.5 rests on the same IEA statement and is reference-only; this row is the one the model reads.</t>
+          <t>Unchanged at 5, so the central case is untouched by the 3 September 2026 band change. Applied to pre-FID headline assets. Two exceptions from 27 September 2026 (decisions: Freddie). (1) Not added where the register's first_export_year_assumes_fid is True, because the developer date already allows for the build after an FID: Ksi Lisims (2032) and Tilbury Phase 1b (2031). (2) Where an asset's life comes from project_life_years with no licence end and no authorised term (Fermeuse 18 years, Summit Lake 30 years), the delay moves the whole life later instead of cutting its last years; the Monte Carlo does the same draw by draw. post_fid_to_completion = 4.5 rests on the same IEA statement and is reference-only; this row is the one the model reads.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -3383,7 +3384,7 @@
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>Figure-8 appendix counterfactual and Emission Factors range_low. NOT used in the central case, which is gas turbine 0.29 for every terminal. BC EAO 0.021 grid / 0.156 gas-barge are a separate SI sensitivity on a facility-total boundary.</t>
+          <t>Electric-drive sensitivity (src/drive_sensitivity.py): every headline terminal on electric drive at this figure, against the all-gas central (decision 27 Sep 2026). Also the section 9 electrification appendix. No longer Emission Factors range_low, which is 0.26 (gas-turbine plants only) from 27 Sep 2026. NOT used in the central case, which is gas turbine 0.29 for every terminal.</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4359,7 +4360,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>SENSITIVITY ONLY - the central liquefaction factor stays 0.29 for every terminal. BOUNDARY: this is the facility total intensity including marine sources, not the liquefaction stage alone, so it is not like for like with the 0.29 liquefaction factor on the Emission Factors sheet. Any comparison against 0.29 is therefore approximate and is labelled as such wherever it is reported.</t>
+          <t>SENSITIVITY ONLY - the central liquefaction factor stays 0.29 for every terminal. Used as the best case in the all-electric drive sensitivity (src/drive_sensitivity.py, decision 27 Sep 2026). BOUNDARY: this is the facility total intensity including marine sources, not the liquefaction stage alone, so it is not like for like with the 0.29 liquefaction factor on the Emission Factors sheet. Any comparison against 0.29 is therefore approximate and is labelled as such wherever it is reported.</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -5028,7 +5029,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>CER may issue LNG licences up to 50 years.</t>
+          <t>50 years is the legal maximum term for a CER LNG export licence since Bill C-15 received royal assent on 26 March 2026. Source: Major Projects Office, LNG Canada Phase 2: https://www.canada.ca/en/privy-council/major-projects-office/projects/national/lng-canada.html</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr"/>
@@ -5206,6 +5207,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -5406,7 +5408,7 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>79.6 mtpa (14.0 operating, 5.4 under construction, 60.2 proposed)</t>
+          <t>85.55 mtpa (14.0 operating, 5.85 under construction, 65.7 proposed; asset register of 27 Sep 2026)</t>
         </is>
       </c>
       <c r="P2" s="4" t="inlineStr">
@@ -6116,7 +6118,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>high - would lower liquefaction by about 80 percent if applied to the whole slate</t>
+          <t>high - would lower liquefaction by about half at 0.15, or by over 90 percent at the 0.021 grid best case, if applied to the whole slate. The all-electric sensitivity in src/drive_sensitivity.py puts a number on it.</t>
         </is>
       </c>
     </row>
@@ -6187,32 +6189,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>liquefaction_electric 0.12</t>
+          <t>liquefaction_electric (was 0.12)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Parameters:liquefaction_electric; Emission Factors range_low</t>
+          <t>Parameters:liquefaction_electric</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>assumption, declared</t>
+          <t>RESOLVED</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>No Pembina document stating 0.12 tCO2e/t was located.</t>
+          <t>0.12 replaced by 0.15 on 3 Sep 2026 (Pembina Institute, Gorski and Lam 2023, https://www.pembina.org/reports/squaring-the-circle-state-of-lng-2023.pdf). From 27 Sep 2026 it is no longer Emission Factors range_low (now 0.26, Delphi Group 2013, https://www2.gov.bc.ca/assets/gov/environment/climate-change/ind/lng/lng_emissions_benchmarking_-_march_2013.pdf); it drives the all-electric sensitivity only.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>A Pembina table, or replacement by the EAO 0.021/0.156 pair as the electric counterfactual.</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>low - not used in the central case</t>
+          <t>closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add figure 2(c): annual emissions by territory against Canada's target pathway
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Data_Inputs.xlsx
+++ b/Inputs/Canada_LNG_Data_Inputs.xlsx
@@ -1047,7 +1047,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
@@ -2475,12 +2474,12 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>REFERENCE-ONLY. Read by no module. The government's own projection of where 2030 emissions actually land, against a target of 417-455. Kept because it is the evidence for the statement that Canada is not on track. LIVE COUNTERPART: canada_2030_overshoot_gap = 200, which is the figure the model reads for the overshoot line.</t>
+          <t>LIVE. Read by src/figures_report.py figure_2c_territorial_trajectory as the projected 2030 emissions under current policy, the single marker on Figure 2(c). The government's own projection of where 2030 emissions actually land, against a target of 417-455, and the evidence that Canada is not on track. canada_2030_overshoot_gap = 200 remains the overshoot line.</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>reference-only</t>
+          <t>live</t>
         </is>
       </c>
     </row>
@@ -5207,7 +5206,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Revise figure 2(c): crossover dots and year lines, drop the 2030 projection
</commit_message>
<xml_diff>
--- a/Inputs/Canada_LNG_Data_Inputs.xlsx
+++ b/Inputs/Canada_LNG_Data_Inputs.xlsx
@@ -2474,12 +2474,12 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>LIVE. Read by src/figures_report.py figure_2c_territorial_trajectory as the projected 2030 emissions under current policy, the single marker on Figure 2(c). The government's own projection of where 2030 emissions actually land, against a target of 417-455, and the evidence that Canada is not on track. canada_2030_overshoot_gap = 200 remains the overshoot line.</t>
+          <t>REFERENCE-ONLY. Read by no module. The government's own projection of where 2030 emissions actually land, against a target of 417-455. Kept because it is the evidence for the statement that Canada is not on track. LIVE COUNTERPART: canada_2030_overshoot_gap = 200, which is the figure the model reads for the overshoot line. Read by no module (removed from figure 2(c) on 28 Sep 2026).</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>reference-only</t>
         </is>
       </c>
     </row>

</xml_diff>